<commit_message>
Paruosti 3 skriptai duomenu tvarkymui
</commit_message>
<xml_diff>
--- a/0_SELECT_ZIVE_DATA_2023/AnotacijosLogai/07_Anotacijos_logai/07_Anotavimo_logas.xlsx
+++ b/0_SELECT_ZIVE_DATA_2023/AnotacijosLogai/07_Anotacijos_logai/07_Anotavimo_logas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kesju\DI\2025_ZIVEO\PROJECT_TRAIN_UNET\0_SELECT_ZIVE_DATA_2023\AnotacijosLogai\07_Anotacijos_logai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B983BE5-01C3-4394-993A-C231E4E65FBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D50DD690-A110-4983-A508-9761CA6963BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1900" windowWidth="19200" windowHeight="7710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="logas" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="63">
   <si>
     <t>basename</t>
   </si>
@@ -219,6 +219,12 @@
   </si>
   <si>
     <t>Nika</t>
+  </si>
+  <si>
+    <t>1643055.090</t>
+  </si>
+  <si>
+    <t>1086_4</t>
   </si>
 </sst>
 </file>
@@ -251,7 +257,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -264,8 +270,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -288,11 +300,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -315,6 +338,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -595,10 +622,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:U12"/>
+  <dimension ref="A1:U13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.90625" customWidth="1"/>
     <col min="3" max="3" width="13.81640625" customWidth="1"/>
     <col min="4" max="4" width="10.81640625" bestFit="1" customWidth="1"/>
@@ -1032,6 +1059,26 @@
         <v>60</v>
       </c>
     </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A13" s="8">
+        <v>12</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D13" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:M1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: update annotation logs with additional noise timestamps and remove temporary files
</commit_message>
<xml_diff>
--- a/0_SELECT_ZIVE_DATA_2023/AnotacijosLogai/07_Anotacijos_logai/07_Anotavimo_logas.xlsx
+++ b/0_SELECT_ZIVE_DATA_2023/AnotacijosLogai/07_Anotacijos_logai/07_Anotavimo_logas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kesju\DI\2025_ZIVEO\PROJECT_TRAIN_UNET\0_SELECT_ZIVE_DATA_2023\AnotacijosLogai\07_Anotacijos_logai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91B41135-962E-4EDE-8C4B-D84B68BAC38C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF783B4-0CC7-4055-B1FB-54C13E0D4696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -714,7 +714,9 @@
         <v>60</v>
       </c>
       <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
+      <c r="I2" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="J2" s="4"/>
       <c r="K2" s="6" t="s">
         <v>5</v>
@@ -748,7 +750,9 @@
         <v>60</v>
       </c>
       <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
+      <c r="I3" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="J3" s="4"/>
       <c r="K3" s="6" t="s">
         <v>11</v>
@@ -783,7 +787,9 @@
         <v>60</v>
       </c>
       <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
+      <c r="I4" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="J4" s="4"/>
       <c r="K4" s="6"/>
       <c r="L4" t="s">
@@ -816,7 +822,9 @@
         <v>60</v>
       </c>
       <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
+      <c r="I5" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="J5" s="4"/>
       <c r="K5" s="6" t="s">
         <v>20</v>
@@ -851,7 +859,9 @@
         <v>60</v>
       </c>
       <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
+      <c r="I6" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="J6" s="4"/>
       <c r="K6" s="6" t="s">
         <v>25</v>
@@ -886,7 +896,9 @@
         <v>60</v>
       </c>
       <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
+      <c r="I7" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="J7" s="4"/>
       <c r="K7" s="6" t="s">
         <v>25</v>
@@ -921,7 +933,9 @@
         <v>60</v>
       </c>
       <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
+      <c r="I8" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="J8" s="4"/>
       <c r="K8" s="6" t="s">
         <v>25</v>
@@ -956,7 +970,9 @@
         <v>60</v>
       </c>
       <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
+      <c r="I9" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="J9" s="4"/>
       <c r="K9" s="6" t="s">
         <v>36</v>
@@ -991,7 +1007,9 @@
         <v>60</v>
       </c>
       <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
+      <c r="I10" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="J10" s="4"/>
       <c r="K10" s="6" t="s">
         <v>40</v>
@@ -1025,7 +1043,9 @@
         <v>60</v>
       </c>
       <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
+      <c r="I11" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="J11" s="4"/>
       <c r="K11" s="6" t="s">
         <v>45</v>
@@ -1059,6 +1079,9 @@
       <c r="G12" s="3" t="s">
         <v>60</v>
       </c>
+      <c r="I12" s="4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A13" s="8">
@@ -1078,6 +1101,9 @@
       </c>
       <c r="G13" s="8" t="s">
         <v>60</v>
+      </c>
+      <c r="H13" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>